<commit_message>
content: completar enunciado 4.1.35 y corregir apuntes del programa
Con el enunciado completo, las 107 soluciones quedan válidas y en forma
canónica; la hoja Temas ya referencia los apuntes existentes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Programa.xlsx
+++ b/content/Programa.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29103"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="209" documentId="11_7E4E55BF84DCCEE3ED7FF6F99031F45BFA722949" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AED53456-AE0B-429F-B753-BAD37C92B2B3}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="11_7E4E55BF84DCCEE3ED7FF6F99031F45BFA722949" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F511486-98ED-4D1D-A693-780963701553}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cabecera" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="95">
   <si>
     <t>Materia</t>
   </si>
@@ -51,7 +51,7 @@
     <t>Licenciatura en Ciencias de Datos</t>
   </si>
   <si>
-    <t>["Ricardo Di Pasquale","Alejandro Isidro","Luciana González"]</t>
+    <t>["Ricardo Di Pasquale","Alejandro Isidro","Edgardo Sanchez", "Delfina Las Heras"]</t>
   </si>
   <si>
     <t>Objetivo</t>
@@ -102,7 +102,7 @@
     <t>Apunte Relacionado</t>
   </si>
   <si>
-    <t>["Apunte 1 - Breve introduccion a la gestion de Datos.pdf"]</t>
+    <t>["001 - Clase Teórica #1 - Apunte 1 - Breve introduccion a la gestion de Datos - Parte 1.pdf"]</t>
   </si>
   <si>
     <t>Breve introducción a la gestión de datos</t>
@@ -114,6 +114,9 @@
     <t>Características de un DBMS</t>
   </si>
   <si>
+    <t>["007 - Prep. Fishbowl #1 - Apunte 2 - Breve introduccion a la gestion de Datos - Parte 2.pdf"]</t>
+  </si>
+  <si>
     <t>Perspectiva histórica de los modelos de bases de datos</t>
   </si>
   <si>
@@ -129,6 +132,9 @@
     <t>Tipos de archivos</t>
   </si>
   <si>
+    <t>["011 - Clase Teórica #2 - Almacenamiento fisico.pdf"]</t>
+  </si>
+  <si>
     <t>Manejo de Archivos</t>
   </si>
   <si>
@@ -138,19 +144,19 @@
     <t>Almacenamientos intermedios</t>
   </si>
   <si>
-    <t>Técnicas de dispersión</t>
-  </si>
-  <si>
     <t>Detalles de la Arquitectura de un DBMS respecto de la gestión de Archivos: File Manager, Disk Manager, Cache Manager.</t>
   </si>
   <si>
     <t>Índices</t>
   </si>
   <si>
+    <t>["019 - Apunte de índices.pdf"]</t>
+  </si>
+  <si>
     <t>Tipos de Índices</t>
   </si>
   <si>
-    <t>["Apunte 2 - Introduccion al Modelo Relacional.pdf"]</t>
+    <t>["001 - Clase Teórica #3 - Apunte - Introduccion al Modelo Relacional.pdf"]</t>
   </si>
   <si>
     <t>Modelos jerárquicos y de red</t>
@@ -159,21 +165,15 @@
     <t>Modelo Orientado a Objetos</t>
   </si>
   <si>
-    <t>Modelo Objeto/Relacional</t>
-  </si>
-  <si>
     <t>Algebra relacional: Operaciones, Práctica</t>
   </si>
   <si>
-    <t>["Apunte 3 - Lenguajes relacionales.pdf", "Relational Theory for Computer Professionals - Date - Capitulo4.pdf"]</t>
+    <t>["001 - Taller#3 - Apunte - Lenguajes relacionales.pdf"]</t>
   </si>
   <si>
     <t>Cálculo relacional</t>
   </si>
   <si>
-    <t>["Apunte 3 - Lenguajes relacionales.pdf"]</t>
-  </si>
-  <si>
     <t>Lenguajes relacionalmente completos</t>
   </si>
   <si>
@@ -186,6 +186,9 @@
     <t>Métricas de Ingeniería de Software en Bases de Datos Relacionales</t>
   </si>
   <si>
+    <t>["003 - Clase Teórica #3 - Apunte - Metricas de Bases de Datos relacionales.pdf"]</t>
+  </si>
+  <si>
     <t>Modelo Entidad-Relación</t>
   </si>
   <si>
@@ -210,12 +213,12 @@
     <t>Valoración de las técnicas de normalización como forma canónica</t>
   </si>
   <si>
-    <t>Práctica de diseño normalizado</t>
-  </si>
-  <si>
     <t>Introducción al SQL</t>
   </si>
   <si>
+    <t>["009 - Taller #8 - Visuals - De Algebra Relacional a SQL.pdf"]</t>
+  </si>
+  <si>
     <t>Analogías y diferencias con el álgebra relacional</t>
   </si>
   <si>
@@ -228,7 +231,7 @@
     <t>Vistas</t>
   </si>
   <si>
-    <t>Cursores</t>
+    <t>["013 - Taller #11 - SQL Stored Procedures.pdf"]</t>
   </si>
   <si>
     <t>Stored Procedures</t>
@@ -240,19 +243,22 @@
     <t>Seguridad</t>
   </si>
   <si>
+    <t>["015 - Clase Teórica #6 - Apunte - Seguridad en Bases de Datos.pdf"]</t>
+  </si>
+  <si>
     <t>DCL</t>
   </si>
   <si>
     <t>Planes de ejecución</t>
   </si>
   <si>
-    <t>Implementación física de diseños normalizados en el laboratorio</t>
-  </si>
-  <si>
-    <t>Resolución de problemas de consulta</t>
+    <t>["001 - Clase Teórica #7 - Apunte - Optimización.pdf"]</t>
   </si>
   <si>
     <t>Propiedades ACID</t>
+  </si>
+  <si>
+    <t>["001 - Apunte - Transacciones, Concurrencia y Recuperación.pdf"]</t>
   </si>
   <si>
     <t>Anomalías</t>
@@ -860,7 +866,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64E9A507-868B-4275-97F5-2C636E938BD6}">
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.85546875" bestFit="1" customWidth="1"/>
@@ -897,7 +903,7 @@
       <c r="B3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="E3" t="s">
@@ -912,7 +918,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -920,10 +926,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -931,10 +937,10 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -942,10 +948,10 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -953,10 +959,10 @@
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -964,7 +970,10 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -972,7 +981,10 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -980,6 +992,9 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
         <v>32</v>
       </c>
     </row>
@@ -988,7 +1003,10 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -996,7 +1014,10 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1004,7 +1025,10 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1012,15 +1036,21 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1028,10 +1058,10 @@
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1039,10 +1069,10 @@
         <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1050,10 +1080,10 @@
         <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1061,10 +1091,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1072,10 +1102,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1083,10 +1113,10 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1094,10 +1124,10 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1105,29 +1135,32 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>52</v>
+      </c>
+      <c r="C26" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1135,7 +1168,10 @@
         <v>4</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>53</v>
+      </c>
+      <c r="C27" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1143,7 +1179,10 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="C28" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1151,7 +1190,10 @@
         <v>4</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
+        <v>55</v>
+      </c>
+      <c r="C29" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1159,7 +1201,10 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>53</v>
+        <v>56</v>
+      </c>
+      <c r="C30" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1167,7 +1212,7 @@
         <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1175,303 +1220,342 @@
         <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
+        <v>59</v>
+      </c>
+      <c r="C33" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
+        <v>61</v>
+      </c>
+      <c r="C34" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36">
         <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37">
         <v>5</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+        <v>64</v>
+      </c>
+      <c r="C37" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38">
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+        <v>66</v>
+      </c>
+      <c r="C38" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39">
         <v>5</v>
       </c>
       <c r="B39" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
+        <v>67</v>
+      </c>
+      <c r="C39" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40">
         <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
+        <v>68</v>
+      </c>
+      <c r="C40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41">
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
+        <v>70</v>
+      </c>
+      <c r="C41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42">
         <v>5</v>
       </c>
       <c r="B42" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
+        <v>71</v>
+      </c>
+      <c r="C42" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B43" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2">
+        <v>73</v>
+      </c>
+      <c r="C43" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B44" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2">
+        <v>75</v>
+      </c>
+      <c r="C44" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
+        <v>76</v>
+      </c>
+      <c r="C45" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B46" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2">
+        <v>77</v>
+      </c>
+      <c r="C46" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="A47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2">
+        <v>78</v>
+      </c>
+      <c r="C47" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
+        <v>79</v>
+      </c>
+      <c r="C48" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
       <c r="A49">
         <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
+        <v>80</v>
+      </c>
+      <c r="C49" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50">
         <v>6</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
+        <v>81</v>
+      </c>
+      <c r="C50" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51">
         <v>6</v>
       </c>
       <c r="B51" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:3">
       <c r="A52">
         <v>6</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
+        <v>83</v>
+      </c>
+      <c r="C52" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
+        <v>84</v>
+      </c>
+      <c r="C53" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
       <c r="A54">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B54" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2">
+        <v>85</v>
+      </c>
+      <c r="C54" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
       <c r="A55">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B55" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
+        <v>86</v>
+      </c>
+      <c r="C55" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
       <c r="A56">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B56" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
+        <v>87</v>
+      </c>
+      <c r="C56" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
       <c r="A57">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B57" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
+        <v>88</v>
+      </c>
+      <c r="C57" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
       <c r="A58">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B58" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2">
+        <v>89</v>
+      </c>
+      <c r="C58" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
       <c r="A59">
         <v>7</v>
       </c>
       <c r="B59" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2">
+        <v>90</v>
+      </c>
+      <c r="C59" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
       <c r="A60">
         <v>7</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2">
+        <v>91</v>
+      </c>
+      <c r="C60" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
       <c r="A61">
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2">
+        <v>92</v>
+      </c>
+      <c r="C61" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
       <c r="A62">
         <v>7</v>
       </c>
       <c r="B62" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2">
+        <v>93</v>
+      </c>
+      <c r="C62" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
       <c r="A63">
         <v>7</v>
       </c>
       <c r="B63" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="A64">
-        <v>7</v>
-      </c>
-      <c r="B64" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2">
-      <c r="A65">
-        <v>7</v>
-      </c>
-      <c r="B65" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2">
-      <c r="A66">
-        <v>7</v>
-      </c>
-      <c r="B66" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2">
-      <c r="A67">
-        <v>7</v>
-      </c>
-      <c r="B67" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2">
-      <c r="A68">
-        <v>7</v>
-      </c>
-      <c r="B68" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2">
-      <c r="A69">
-        <v>7</v>
-      </c>
-      <c r="B69" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="C63" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>